<commit_message>
docs: neutralize regulatory applicability wording
Reframe scoped regulatory applicability, satisfaction, and retention-duration assertions as potential triggers, firm-policy examples, or evidence for counsel review while preserving citations and table structure.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -2032,7 +2032,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Configure WORM-immutable retention for records subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior required for WORM compliance</t>
+          <t>Configure WORM-style immutable retention for records the firm identifies as subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior; firms should confirm WORM applicability with counsel</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Increase post-use review sampling rate to 25% of Copilot-assisted communications (FSI-recommended baseline); configure via CC policy &gt; Review percentage in the Purview portal</t>
+          <t>Increase post-use review sampling rate to the firm's approved threshold for Copilot-assisted communications (25% is an FSI policy example; confirm with compliance/legal); configure via CC policy &gt; Review percentage in the Purview portal</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Fix framework-neutral review findings
Restore review-cited control strength while keeping regulatory applicability counsel-confirmed, add section-level applicability notes, and refresh generated checklist artifacts.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -2032,7 +2032,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Configure WORM-style immutable retention for records the firm identifies as subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior; firms should confirm WORM applicability with counsel</t>
+          <t>Configure WORM-style immutable retention for records the firm identifies as subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior; WORM applicability: confirm</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Increase post-use review sampling rate to the firm's approved threshold for Copilot-assisted communications (25% is an FSI policy example; confirm with compliance/legal); configure via CC policy &gt; Review percentage in the Purview portal</t>
+          <t>Increase post-use review sampling rate to the firm's approved threshold for Copilot-assisted communications (default threshold: 25%; adjust to the firm-approved threshold with compliance/legal); configure via CC policy &gt; Review percentage in the Purview portal</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: drift re-verification LANE w5
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -3198,17 +3198,17 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Document the tenant's Cowork access posture: which users/groups have usage-based billing enabled, whether the discovery setting is on, and the approval basis for both decisions</t>
+          <t>Document the tenant's Cowork access posture: which users/groups are in a spending policy that selects Cowork, whether the discovery setting is on, and the approval basis for both decisions</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Manage usage-based billing scope, discovery, model toggles, browser-use toggle, and consumption limits through a documented change register</t>
+          <t>Manage Cowork spending-policy scope, discovery, model toggles, browser-use toggle, and consumption limits through a documented change register</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Require dual approval (technology + compliance) before enabling usage-based billing, discovery, browser use, or the Anthropic/Fable model toggles for any regulated or client-facing population</t>
+          <t>Require dual approval (technology + compliance) before enabling Cowork spending-policy access, discovery, browser use, or Anthropic/model controls for any regulated or client-facing population</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: drift re-verification w1
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1392,7 +1392,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Minimum Chinese Wall implementation — addresses the most critical regulatory separation requirements including the Channel Agent IB limitation</t>
+          <t>Minimum ethical-wall implementation for firms whose approved policy requires segment separation, including explicit handling of the Channel Agent IB limitation</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Full Chinese Wall implementation for large, diversified financial institutions subject to frequent SEC/FINRA examinations. The Channel Agent limitation and compensating controls must appear in the examination package.</t>
+          <t>Full ethical-wall implementation for large, diversified financial institutions subject to frequent examinations. The Channel Agent limitation and compensating controls should appear in the examination package where counsel/compliance determine the cited rules or firm policies apply.</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: drift re-verification w1 (1.6-permission-model-audit, 1.7-sharepoint-advanced-management, 1.8-information-architecture-review, 2.4-information-barriers) (#532)
* docs: drift re-verification w1

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* Fix PR 532 regulatory posture blockers

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

---------

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1392,7 +1392,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Minimum Chinese Wall implementation — addresses the most critical regulatory separation requirements including the Channel Agent IB limitation</t>
+          <t>Minimum ethical-wall implementation for firms whose approved policy requires segment separation, including explicit handling of the Channel Agent IB limitation</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Full Chinese Wall implementation for large, diversified financial institutions subject to frequent SEC/FINRA examinations. The Channel Agent limitation and compensating controls must appear in the examination package.</t>
+          <t>Full ethical-wall implementation for large, diversified financial institutions subject to frequent examinations. The Channel Agent limitation and compensating controls should appear in the examination package where counsel/compliance determine the cited rules or firm policies apply.</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Drift wave 5 updates
Merged after re-review fixes and validation.
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -3198,17 +3198,17 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Document the tenant's Cowork access posture: which users/groups have usage-based billing enabled, whether the discovery setting is on, and the approval basis for both decisions</t>
+          <t>Document the tenant's Cowork access posture: which users/groups are in a spending policy that selects Cowork, whether the discovery setting is on, and the approval basis for both decisions</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Manage usage-based billing scope, discovery, model toggles, browser-use toggle, and consumption limits through a documented change register</t>
+          <t>Manage Cowork spending-policy scope, discovery, model toggles, browser-use toggle, and consumption limits through a documented change register</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Require dual approval (technology + compliance) before enabling usage-based billing, discovery, browser use, or the Anthropic/Fable model toggles for any regulated or client-facing population</t>
+          <t>Require dual approval (technology + compliance) before enabling Cowork spending-policy access, discovery, browser use, or Anthropic/model controls for any regulated or client-facing population</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: refresh Sentinel integration guidance
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Governance Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Governance Dashboard'!$A$4:$I$68</definedName>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Enable the Microsoft 365 data connector in Sentinel</t>
+          <t>Enable the Microsoft Copilot data connector in Sentinel for `CopilotActivity`</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: refresh Sentinel integration guidance (#563)
Part of the documentation freshness program.
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Governance Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Governance Dashboard'!$A$4:$I$68</definedName>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Enable the Microsoft 365 data connector in Sentinel</t>
+          <t>Enable the Microsoft Copilot data connector in Sentinel for `CopilotActivity`</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: re-verify Purview and Defender governance controls (#571)
Re-verification of Purview/Defender governance Controls 2.5, 2.9, 2.10 and playbooks against current Microsoft Learn (Graph alerts v2, IRM indicators, data risk graph retirement, MDCA anomaly detections). Independent review passed on this exact head after four fix rounds.
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1602,17 +1602,17 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Provides visibility into Copilot usage patterns without impacting user experience — essential first step for understanding AI interaction behavior. Agent monitoring alerts provide baseline coverage for agent-involved incidents.</t>
+          <t>Provides initial visibility without assuming unsupported native-client coverage or prompt-level telemetry. Shadow AI review and agent monitoring extend the control beyond first-party Copilot alone.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Active monitoring with real-time alerting — suitable for production FSI Copilot deployments where proactive threat detection is needed. Generative AI catalog and agent anomaly detection extend coverage to Shadow AI and agentic threats.</t>
+          <t>Active monitoring with supported browser-session controls and Shadow AI governance, while reserving Purview audit for Copilot prompt/response evidence.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Full session-level governance with automated response — designed for firms with the highest security monitoring requirements. Agent threat detection and Shadow AI governance satisfy FINRA supervisory obligations for agentic AI.</t>
+          <t>Full session-level governance with stronger enforcement on supported browser surfaces, explicit native-client compensating controls, and documented Shadow AI/agent governance evidence.</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -1644,17 +1644,17 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Provides foundational insider risk detection and agent monitoring — minimum monitoring for Copilot deployment in regulated environments</t>
+          <t>Provides foundational insider risk detection and agent monitoring without assuming that optional Security Copilot agent features are already licensed or approved</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Comprehensive insider risk program incorporating AI-specific indicators and agent governance — suitable for most FSI firms</t>
+          <t>Comprehensive insider risk program incorporating AI-specific indicators, optional triage automation, and agent governance — suitable for most FSI firms</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Full insider risk governance with continuous improvement and agent supervisory coverage — designed for firms with active insider threat programs and board-level risk oversight</t>
+          <t>Full insider risk governance with continuous improvement, explicit preview-feature governance, and board-ready evidence for firms with active insider threat programs</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: re-verify Controls 1.15 and 2.13 (#574)
Claim-level re-verification of Controls 1.15 and 2.13 and playbooks against current Microsoft Learn, plus propagation of the Copilot connector rename and Scout tool-server terminology. Independent exact-head reviews passed after three rounds.
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -1755,7 +1755,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Plugin and Graph Connector Security Governance</t>
+          <t>Plugin and Copilot Connector Security Governance</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Maximum restriction during initial Copilot deployment — eliminates third-party extensibility risk entirely</t>
+          <t>Maximum restriction during initial Copilot deployment — helps reduce third-party extensibility risk</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">

</xml_diff>